<commit_message>
Clear 9 'Human checked' Y flags on rows without a human score
RSI v1-v3 and v5-v10 were marked Y with no human fidelity score. Only those
nine Results!O cells changed; Summary values are unchanged (10 rows human-scored,
mean gap 0.2, exact agreement 0.8).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/QC_Eval_Prompt_Error_Sheet.xlsx
+++ b/src/QC_Eval_Prompt_Error_Sheet.xlsx
@@ -2464,9 +2464,7 @@
       <c r="L3" s="10"/>
       <c r="M3" s="10"/>
       <c r="N3" s="10"/>
-      <c r="O3" s="12" t="s">
-        <v>66</v>
-      </c>
+      <c r="O3" s="12"/>
       <c r="P3" s="12"/>
       <c r="Q3" s="11"/>
     </row>
@@ -2495,9 +2493,7 @@
       <c r="L4" s="10"/>
       <c r="M4" s="10"/>
       <c r="N4" s="10"/>
-      <c r="O4" s="12" t="s">
-        <v>66</v>
-      </c>
+      <c r="O4" s="12"/>
       <c r="P4" s="12"/>
       <c r="Q4" s="11"/>
     </row>
@@ -2526,9 +2522,7 @@
       <c r="L5" s="10"/>
       <c r="M5" s="10"/>
       <c r="N5" s="10"/>
-      <c r="O5" s="12" t="s">
-        <v>66</v>
-      </c>
+      <c r="O5" s="12"/>
       <c r="P5" s="12"/>
       <c r="Q5" s="11"/>
     </row>
@@ -2598,9 +2592,7 @@
       <c r="L7" s="10"/>
       <c r="M7" s="10"/>
       <c r="N7" s="10"/>
-      <c r="O7" s="12" t="s">
-        <v>66</v>
-      </c>
+      <c r="O7" s="12"/>
       <c r="P7" s="12"/>
       <c r="Q7" s="11"/>
     </row>
@@ -2629,9 +2621,7 @@
       <c r="L8" s="10"/>
       <c r="M8" s="10"/>
       <c r="N8" s="10"/>
-      <c r="O8" s="12" t="s">
-        <v>66</v>
-      </c>
+      <c r="O8" s="12"/>
       <c r="P8" s="12"/>
       <c r="Q8" s="11"/>
     </row>
@@ -2660,9 +2650,7 @@
       <c r="L9" s="10"/>
       <c r="M9" s="10"/>
       <c r="N9" s="10"/>
-      <c r="O9" s="12" t="s">
-        <v>66</v>
-      </c>
+      <c r="O9" s="12"/>
       <c r="P9" s="12"/>
       <c r="Q9" s="11"/>
     </row>
@@ -2691,9 +2679,7 @@
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
       <c r="N10" s="10"/>
-      <c r="O10" s="12" t="s">
-        <v>66</v>
-      </c>
+      <c r="O10" s="12"/>
       <c r="P10" s="12"/>
       <c r="Q10" s="11"/>
     </row>
@@ -2722,9 +2708,7 @@
       <c r="L11" s="10"/>
       <c r="M11" s="10"/>
       <c r="N11" s="10"/>
-      <c r="O11" s="12" t="s">
-        <v>66</v>
-      </c>
+      <c r="O11" s="12"/>
       <c r="P11" s="12"/>
       <c r="Q11" s="11"/>
     </row>
@@ -2753,9 +2737,7 @@
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
       <c r="N12" s="10"/>
-      <c r="O12" s="12" t="s">
-        <v>66</v>
-      </c>
+      <c r="O12" s="12"/>
       <c r="P12" s="12"/>
       <c r="Q12" s="11"/>
     </row>

</xml_diff>